<commit_message>
chore: update WARN dataset
</commit_message>
<xml_diff>
--- a/data/warn_report.xlsx
+++ b/data/warn_report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://edd.sharepoint.com/sites/WSB-COWSD-380-PCU/Shared Documents/Website Management/3. Webpage Updates/Layoff Services WARN/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{977414B1-1E03-445E-9029-4301A02576F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{A7495394-9A74-42A0-94C1-0B5D11A7B8DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6D5322B-EBF1-45A9-80D2-DE191EF33EDD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="751" xr2:uid="{3EA4B9A5-CE9D-4ACF-B45F-4158810915D4}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="434">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="452">
   <si>
     <t>County/Parish</t>
   </si>
@@ -1229,9 +1229,6 @@
     <t>822 S. Robertson Suite #200  Los Angeles CA 90035</t>
   </si>
   <si>
-    <t>Relocation Permanent</t>
-  </si>
-  <si>
     <t>John Muir Physician Network - 5860 Owens Drive</t>
   </si>
   <si>
@@ -1386,6 +1383,42 @@
   </si>
   <si>
     <t>200 N. Pacific Coast Highway, Suite 300  El Segundo CA 90245</t>
+  </si>
+  <si>
+    <t>Renewal by Andersen LLC</t>
+  </si>
+  <si>
+    <t>18700 Crenshaw Blvd  Torrance CA 90504</t>
+  </si>
+  <si>
+    <t>PayPal</t>
+  </si>
+  <si>
+    <t>2211 N. First Street  San Jose CA 95131</t>
+  </si>
+  <si>
+    <t>22982 Alcalde Drive, Suite 100  Laguna Hills CA 92653</t>
+  </si>
+  <si>
+    <t>Clarmil Manufacturing Corporation</t>
+  </si>
+  <si>
+    <t>30865 San Clemente Street  Hayward CA 94544</t>
+  </si>
+  <si>
+    <t>Arsenal Biosciences, Inc.</t>
+  </si>
+  <si>
+    <t>329 Oyster Point Blvd  South San Francisco CA 94080</t>
+  </si>
+  <si>
+    <t>654 N Harington Dr.  Orange CA 92868</t>
+  </si>
+  <si>
+    <t>Foundation for California Community Colleges</t>
+  </si>
+  <si>
+    <t>1102 Q Street, Suite 4800  Sacramento CA 95811</t>
   </si>
   <si>
     <r>
@@ -1407,7 +1440,7 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-01/01/2023 - 09/02/2026
+01/01/2023 - 09/07/2026
 </t>
     </r>
     <r>
@@ -1421,40 +1454,61 @@
     </r>
   </si>
   <si>
-    <t>Renewal by Andersen LLC</t>
-  </si>
-  <si>
-    <t>18700 Crenshaw Blvd  Torrance CA 90504</t>
-  </si>
-  <si>
-    <t>PayPal</t>
-  </si>
-  <si>
-    <t>2211 N. First Street  San Jose CA 95131</t>
-  </si>
-  <si>
-    <t>22982 Alcalde Drive, Suite 100  Laguna Hills CA 92653</t>
-  </si>
-  <si>
-    <t>Clarmil Manufacturing Corporation</t>
-  </si>
-  <si>
-    <t>30865 San Clemente Street  Hayward CA 94544</t>
-  </si>
-  <si>
-    <t>Arsenal Biosciences, Inc.</t>
-  </si>
-  <si>
-    <t>329 Oyster Point Blvd  South San Francisco CA 94080</t>
-  </si>
-  <si>
-    <t>654 N Harington Dr.  Orange CA 92868</t>
-  </si>
-  <si>
-    <t>Foundation for California Community Colleges</t>
-  </si>
-  <si>
-    <t>1102 Q Street, Suite 4800  Sacramento CA 95811</t>
+    <t>San Luis Obispo County</t>
+  </si>
+  <si>
+    <t>Ventana Grill</t>
+  </si>
+  <si>
+    <t>2575 Price Street  Pismo Beach CA 93449</t>
+  </si>
+  <si>
+    <t>OVG Hospitality</t>
+  </si>
+  <si>
+    <t>10 W. Harbor Boulevard  Ventura CA 93001</t>
+  </si>
+  <si>
+    <t>Homeless Health Care Los Angeles - Crocker Street</t>
+  </si>
+  <si>
+    <t>442 Crocker Street  Los Angeles CA 90013</t>
+  </si>
+  <si>
+    <t>Homeless Health Care Los Angeles - Maple Ave.</t>
+  </si>
+  <si>
+    <t>655 Maple Ave.  Los Angeles CA 90014</t>
+  </si>
+  <si>
+    <t>Homeless Health Care Los Angeles - 2nd Street</t>
+  </si>
+  <si>
+    <t>1282 W 2nd Street  Los Angeles CA 90026</t>
+  </si>
+  <si>
+    <t>Grain Craft, LLC</t>
+  </si>
+  <si>
+    <t>8790 Rochester Ave # B  Rancho Cucamonga CA 91730</t>
+  </si>
+  <si>
+    <t>SonTek (Xylem, Inc.)</t>
+  </si>
+  <si>
+    <t>9940 Summers Ridge Rd.  San Diego CA 92121</t>
+  </si>
+  <si>
+    <t>Eggo Company dba Kellanova</t>
+  </si>
+  <si>
+    <t>475 Eggo Way  San Jose CA 95116</t>
+  </si>
+  <si>
+    <t>Ruiz Food Products, Inc.</t>
+  </si>
+  <si>
+    <t>501 South Alta Avenue  Dinuba CA 93618</t>
   </si>
   <si>
     <r>
@@ -1468,7 +1522,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>07/01/26 to 09/02/2026</t>
+      <t>07/01/26 to 09/07/2026</t>
     </r>
     <r>
       <rPr>
@@ -1488,7 +1542,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>A detailed WARN summary by county and filtered according to processed date. Table Spans cells A2 through I194.</t>
+      <t>A detailed WARN summary by county and filtered according to processed date. Table Spans cells A2 through I203.</t>
     </r>
   </si>
 </sst>
@@ -1603,7 +1657,6 @@
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -2655,8 +2708,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1F69E8FD-21FF-4B81-951D-D7EC70F8E5F9}" name="DetailedWarnReport" displayName="DetailedWarnReport" ref="A2:I194" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
-  <autoFilter ref="A2:I194" xr:uid="{1F69E8FD-21FF-4B81-951D-D7EC70F8E5F9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1F69E8FD-21FF-4B81-951D-D7EC70F8E5F9}" name="DetailedWarnReport" displayName="DetailedWarnReport" ref="A2:I203" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
+  <autoFilter ref="A2:I203" xr:uid="{1F69E8FD-21FF-4B81-951D-D7EC70F8E5F9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:I42">
     <sortCondition ref="C2:C42"/>
   </sortState>
@@ -3077,7 +3130,7 @@
       </c>
       <c r="B3" s="11">
         <f>SUM('Detailed WARN Report '!G:G)</f>
-        <v>10304</v>
+        <v>10975</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3086,7 +3139,7 @@
       </c>
       <c r="B4" s="11">
         <f>COUNTIF('Detailed WARN Report '!F:F,"Layoff Permanent")</f>
-        <v>134</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3113,7 +3166,7 @@
       </c>
       <c r="B7" s="11">
         <f>COUNTIF('Detailed WARN Report '!F:F,"Closure Permanent")</f>
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3122,7 +3175,7 @@
       </c>
       <c r="B8" s="11">
         <f>COUNTIF('Detailed WARN Report '!F:F,"Closure Temporary")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3145,7 +3198,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3E7117B-AC46-45AC-B2F3-AE611FA82488}">
-  <dimension ref="A1:I194"/>
+  <dimension ref="A1:I203"/>
   <sheetFormatPr defaultColWidth="161.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.28515625" style="3" bestFit="1" customWidth="1"/>
@@ -3153,7 +3206,7 @@
     <col min="3" max="3" width="12.140625" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.28515625" style="8" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="45.85546875" style="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.140625" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="50.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="51.85546875" style="3" bestFit="1" customWidth="1"/>
@@ -3166,7 +3219,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="102" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>433</v>
+        <v>451</v>
       </c>
       <c r="E1" s="3"/>
     </row>
@@ -7218,7 +7271,7 @@
         <v>338</v>
       </c>
       <c r="F141" s="28" t="s">
-        <v>367</v>
+        <v>6</v>
       </c>
       <c r="G141" s="30">
         <v>73</v>
@@ -7708,7 +7761,7 @@
         <v>46323</v>
       </c>
       <c r="E158" s="28" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="F158" s="28" t="s">
         <v>6</v>
@@ -7717,7 +7770,7 @@
         <v>1</v>
       </c>
       <c r="H158" s="30" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="I158" s="32" t="s">
         <v>45</v>
@@ -7737,7 +7790,7 @@
         <v>46323</v>
       </c>
       <c r="E159" s="28" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="F159" s="28" t="s">
         <v>6</v>
@@ -7746,7 +7799,7 @@
         <v>23</v>
       </c>
       <c r="H159" s="30" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="I159" s="32" t="s">
         <v>45</v>
@@ -7766,7 +7819,7 @@
         <v>46323</v>
       </c>
       <c r="E160" s="28" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="F160" s="28" t="s">
         <v>6</v>
@@ -7775,7 +7828,7 @@
         <v>4</v>
       </c>
       <c r="H160" s="30" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="I160" s="32" t="s">
         <v>45</v>
@@ -7795,7 +7848,7 @@
         <v>46323</v>
       </c>
       <c r="E161" s="28" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F161" s="28" t="s">
         <v>6</v>
@@ -7804,7 +7857,7 @@
         <v>15</v>
       </c>
       <c r="H161" s="30" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="I161" s="32" t="s">
         <v>45</v>
@@ -7824,7 +7877,7 @@
         <v>46323</v>
       </c>
       <c r="E162" s="28" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="F162" s="28" t="s">
         <v>6</v>
@@ -7833,7 +7886,7 @@
         <v>2</v>
       </c>
       <c r="H162" s="30" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="I162" s="32" t="s">
         <v>45</v>
@@ -7853,7 +7906,7 @@
         <v>46323</v>
       </c>
       <c r="E163" s="28" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="F163" s="28" t="s">
         <v>6</v>
@@ -7862,7 +7915,7 @@
         <v>15</v>
       </c>
       <c r="H163" s="30" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="I163" s="32" t="s">
         <v>45</v>
@@ -7882,7 +7935,7 @@
         <v>46323</v>
       </c>
       <c r="E164" s="28" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="F164" s="28" t="s">
         <v>6</v>
@@ -7891,7 +7944,7 @@
         <v>3</v>
       </c>
       <c r="H164" s="30" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="I164" s="32" t="s">
         <v>45</v>
@@ -7911,7 +7964,7 @@
         <v>46323</v>
       </c>
       <c r="E165" s="28" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F165" s="28" t="s">
         <v>6</v>
@@ -7920,7 +7973,7 @@
         <v>2</v>
       </c>
       <c r="H165" s="30" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="I165" s="32" t="s">
         <v>45</v>
@@ -7940,7 +7993,7 @@
         <v>46323</v>
       </c>
       <c r="E166" s="28" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F166" s="28" t="s">
         <v>6</v>
@@ -7949,7 +8002,7 @@
         <v>1</v>
       </c>
       <c r="H166" s="30" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="I166" s="32" t="s">
         <v>45</v>
@@ -7969,7 +8022,7 @@
         <v>46323</v>
       </c>
       <c r="E167" s="28" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F167" s="28" t="s">
         <v>6</v>
@@ -7978,7 +8031,7 @@
         <v>2</v>
       </c>
       <c r="H167" s="30" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="I167" s="32" t="s">
         <v>45</v>
@@ -7998,7 +8051,7 @@
         <v>46323</v>
       </c>
       <c r="E168" s="28" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="F168" s="28" t="s">
         <v>6</v>
@@ -8007,7 +8060,7 @@
         <v>6</v>
       </c>
       <c r="H168" s="30" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="I168" s="32" t="s">
         <v>45</v>
@@ -8027,7 +8080,7 @@
         <v>46323</v>
       </c>
       <c r="E169" s="28" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="F169" s="28" t="s">
         <v>6</v>
@@ -8036,7 +8089,7 @@
         <v>1</v>
       </c>
       <c r="H169" s="30" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="I169" s="32" t="s">
         <v>45</v>
@@ -8056,7 +8109,7 @@
         <v>46323</v>
       </c>
       <c r="E170" s="28" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="F170" s="28" t="s">
         <v>6</v>
@@ -8065,7 +8118,7 @@
         <v>1</v>
       </c>
       <c r="H170" s="30" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I170" s="32" t="s">
         <v>45</v>
@@ -8085,7 +8138,7 @@
         <v>46323</v>
       </c>
       <c r="E171" s="28" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="F171" s="28" t="s">
         <v>6</v>
@@ -8094,7 +8147,7 @@
         <v>1</v>
       </c>
       <c r="H171" s="30" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="I171" s="32" t="s">
         <v>45</v>
@@ -8114,7 +8167,7 @@
         <v>46323</v>
       </c>
       <c r="E172" s="28" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="F172" s="28" t="s">
         <v>6</v>
@@ -8123,7 +8176,7 @@
         <v>1</v>
       </c>
       <c r="H172" s="30" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="I172" s="32" t="s">
         <v>45</v>
@@ -8143,7 +8196,7 @@
         <v>46318</v>
       </c>
       <c r="E173" s="28" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="F173" s="28" t="s">
         <v>6</v>
@@ -8152,7 +8205,7 @@
         <v>7</v>
       </c>
       <c r="H173" s="30" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="I173" s="32" t="s">
         <v>34</v>
@@ -8172,7 +8225,7 @@
         <v>46329</v>
       </c>
       <c r="E174" s="28" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F174" s="28" t="s">
         <v>52</v>
@@ -8181,7 +8234,7 @@
         <v>51</v>
       </c>
       <c r="H174" s="30" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="I174" s="32" t="s">
         <v>36</v>
@@ -8201,7 +8254,7 @@
         <v>46328</v>
       </c>
       <c r="E175" s="28" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F175" s="28" t="s">
         <v>6</v>
@@ -8210,7 +8263,7 @@
         <v>79</v>
       </c>
       <c r="H175" s="30" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="I175" s="32" t="s">
         <v>45</v>
@@ -8230,7 +8283,7 @@
         <v>46328</v>
       </c>
       <c r="E176" s="28" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="F176" s="28" t="s">
         <v>6</v>
@@ -8239,7 +8292,7 @@
         <v>16</v>
       </c>
       <c r="H176" s="30" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="I176" s="32" t="s">
         <v>45</v>
@@ -8288,7 +8341,7 @@
         <v>46332</v>
       </c>
       <c r="E178" s="28" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="F178" s="28" t="s">
         <v>52</v>
@@ -8297,7 +8350,7 @@
         <v>189</v>
       </c>
       <c r="H178" s="30" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="I178" s="32" t="s">
         <v>41</v>
@@ -8317,7 +8370,7 @@
         <v>46324</v>
       </c>
       <c r="E179" s="28" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F179" s="28" t="s">
         <v>6</v>
@@ -8326,7 +8379,7 @@
         <v>23</v>
       </c>
       <c r="H179" s="30" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="I179" s="32" t="s">
         <v>45</v>
@@ -8346,7 +8399,7 @@
         <v>46324</v>
       </c>
       <c r="E180" s="28" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="F180" s="28" t="s">
         <v>6</v>
@@ -8355,7 +8408,7 @@
         <v>16</v>
       </c>
       <c r="H180" s="30" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="I180" s="32" t="s">
         <v>45</v>
@@ -8375,7 +8428,7 @@
         <v>46324</v>
       </c>
       <c r="E181" s="28" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F181" s="28" t="s">
         <v>6</v>
@@ -8384,7 +8437,7 @@
         <v>16</v>
       </c>
       <c r="H181" s="30" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="I181" s="32" t="s">
         <v>45</v>
@@ -8404,7 +8457,7 @@
         <v>46324</v>
       </c>
       <c r="E182" s="28" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F182" s="28" t="s">
         <v>6</v>
@@ -8413,7 +8466,7 @@
         <v>13</v>
       </c>
       <c r="H182" s="30" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="I182" s="32" t="s">
         <v>45</v>
@@ -8433,7 +8486,7 @@
         <v>46295</v>
       </c>
       <c r="E183" s="28" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F183" s="28" t="s">
         <v>6</v>
@@ -8442,7 +8495,7 @@
         <v>28</v>
       </c>
       <c r="H183" s="30" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="I183" s="32" t="s">
         <v>41</v>
@@ -8462,7 +8515,7 @@
         <v>46315</v>
       </c>
       <c r="E184" s="28" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F184" s="28" t="s">
         <v>6</v>
@@ -8471,7 +8524,7 @@
         <v>70</v>
       </c>
       <c r="H184" s="30" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="I184" s="32" t="s">
         <v>41</v>
@@ -8491,7 +8544,7 @@
         <v>46372</v>
       </c>
       <c r="E185" s="28" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F185" s="28" t="s">
         <v>6</v>
@@ -8500,7 +8553,7 @@
         <v>128</v>
       </c>
       <c r="H185" s="30" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I185" s="32" t="s">
         <v>38</v>
@@ -8520,7 +8573,7 @@
         <v>46315</v>
       </c>
       <c r="E186" s="28" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F186" s="28" t="s">
         <v>6</v>
@@ -8529,7 +8582,7 @@
         <v>78</v>
       </c>
       <c r="H186" s="30" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="I186" s="32" t="s">
         <v>41</v>
@@ -8549,7 +8602,7 @@
         <v>46280</v>
       </c>
       <c r="E187" s="28" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="F187" s="28" t="s">
         <v>6</v>
@@ -8558,7 +8611,7 @@
         <v>738</v>
       </c>
       <c r="H187" s="30" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="I187" s="32" t="s">
         <v>45</v>
@@ -8578,7 +8631,7 @@
         <v>46325</v>
       </c>
       <c r="E188" s="28" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="F188" s="28" t="s">
         <v>52</v>
@@ -8587,7 +8640,7 @@
         <v>108</v>
       </c>
       <c r="H188" s="30" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="I188" s="32" t="s">
         <v>34</v>
@@ -8607,7 +8660,7 @@
         <v>46324</v>
       </c>
       <c r="E189" s="28" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="F189" s="28" t="s">
         <v>6</v>
@@ -8616,7 +8669,7 @@
         <v>58</v>
       </c>
       <c r="H189" s="30" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="I189" s="32" t="s">
         <v>41</v>
@@ -8636,7 +8689,7 @@
         <v>46325</v>
       </c>
       <c r="E190" s="28" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="F190" s="28" t="s">
         <v>6</v>
@@ -8645,7 +8698,7 @@
         <v>251</v>
       </c>
       <c r="H190" s="30" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="I190" s="32" t="s">
         <v>39</v>
@@ -8665,7 +8718,7 @@
         <v>46328</v>
       </c>
       <c r="E191" s="28" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="F191" s="28" t="s">
         <v>6</v>
@@ -8674,7 +8727,7 @@
         <v>153</v>
       </c>
       <c r="H191" s="30" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="I191" s="32" t="s">
         <v>34</v>
@@ -8694,7 +8747,7 @@
         <v>46328</v>
       </c>
       <c r="E192" s="28" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="F192" s="28" t="s">
         <v>6</v>
@@ -8703,7 +8756,7 @@
         <v>79</v>
       </c>
       <c r="H192" s="30" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="I192" s="32" t="s">
         <v>34</v>
@@ -8723,7 +8776,7 @@
         <v>46328</v>
       </c>
       <c r="E193" s="28" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="F193" s="28" t="s">
         <v>6</v>
@@ -8732,7 +8785,7 @@
         <v>52</v>
       </c>
       <c r="H193" s="30" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="I193" s="32" t="s">
         <v>34</v>
@@ -8752,7 +8805,7 @@
         <v>46325</v>
       </c>
       <c r="E194" s="28" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F194" s="28" t="s">
         <v>6</v>
@@ -8761,10 +8814,271 @@
         <v>178</v>
       </c>
       <c r="H194" s="30" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="I194" s="32" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A195" s="28" t="s">
+        <v>432</v>
+      </c>
+      <c r="B195" s="29">
+        <v>46267</v>
+      </c>
+      <c r="C195" s="29">
+        <v>46268</v>
+      </c>
+      <c r="D195" s="29">
+        <v>46283</v>
+      </c>
+      <c r="E195" s="28" t="s">
+        <v>433</v>
+      </c>
+      <c r="F195" s="28" t="s">
+        <v>101</v>
+      </c>
+      <c r="G195" s="30">
+        <v>82</v>
+      </c>
+      <c r="H195" s="30" t="s">
+        <v>434</v>
+      </c>
+      <c r="I195" s="32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A196" s="28" t="s">
+        <v>326</v>
+      </c>
+      <c r="B196" s="29">
+        <v>46268</v>
+      </c>
+      <c r="C196" s="29">
+        <v>46268</v>
+      </c>
+      <c r="D196" s="29">
+        <v>46341</v>
+      </c>
+      <c r="E196" s="28" t="s">
+        <v>435</v>
+      </c>
+      <c r="F196" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="G196" s="30">
+        <v>128</v>
+      </c>
+      <c r="H196" s="30" t="s">
+        <v>436</v>
+      </c>
+      <c r="I196" s="32" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A197" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="B197" s="29">
+        <v>46267</v>
+      </c>
+      <c r="C197" s="29">
+        <v>46269</v>
+      </c>
+      <c r="D197" s="29">
+        <v>46329</v>
+      </c>
+      <c r="E197" s="28" t="s">
+        <v>437</v>
+      </c>
+      <c r="F197" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="G197" s="30">
+        <v>117</v>
+      </c>
+      <c r="H197" s="30" t="s">
+        <v>438</v>
+      </c>
+      <c r="I197" s="32" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A198" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="B198" s="29">
+        <v>46267</v>
+      </c>
+      <c r="C198" s="29">
+        <v>46269</v>
+      </c>
+      <c r="D198" s="29">
+        <v>46329</v>
+      </c>
+      <c r="E198" s="28" t="s">
+        <v>439</v>
+      </c>
+      <c r="F198" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="G198" s="30">
+        <v>16</v>
+      </c>
+      <c r="H198" s="30" t="s">
+        <v>440</v>
+      </c>
+      <c r="I198" s="32" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A199" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="B199" s="29">
+        <v>46267</v>
+      </c>
+      <c r="C199" s="29">
+        <v>46269</v>
+      </c>
+      <c r="D199" s="29">
+        <v>46329</v>
+      </c>
+      <c r="E199" s="28" t="s">
+        <v>441</v>
+      </c>
+      <c r="F199" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="G199" s="30">
+        <v>1</v>
+      </c>
+      <c r="H199" s="30" t="s">
+        <v>442</v>
+      </c>
+      <c r="I199" s="32" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A200" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="B200" s="29">
+        <v>46266</v>
+      </c>
+      <c r="C200" s="29">
+        <v>46269</v>
+      </c>
+      <c r="D200" s="29">
+        <v>46325</v>
+      </c>
+      <c r="E200" s="28" t="s">
+        <v>443</v>
+      </c>
+      <c r="F200" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="G200" s="30">
+        <v>3</v>
+      </c>
+      <c r="H200" s="30" t="s">
+        <v>444</v>
+      </c>
+      <c r="I200" s="32" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="201" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A201" s="28" t="s">
+        <v>207</v>
+      </c>
+      <c r="B201" s="29">
+        <v>46269</v>
+      </c>
+      <c r="C201" s="29">
+        <v>46269</v>
+      </c>
+      <c r="D201" s="29">
+        <v>46332</v>
+      </c>
+      <c r="E201" s="28" t="s">
+        <v>445</v>
+      </c>
+      <c r="F201" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="G201" s="30">
+        <v>36</v>
+      </c>
+      <c r="H201" s="30" t="s">
+        <v>446</v>
+      </c>
+      <c r="I201" s="32" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A202" s="28" t="s">
+        <v>103</v>
+      </c>
+      <c r="B202" s="29">
+        <v>46269</v>
+      </c>
+      <c r="C202" s="29">
+        <v>46269</v>
+      </c>
+      <c r="D202" s="29">
+        <v>46330</v>
+      </c>
+      <c r="E202" s="28" t="s">
+        <v>447</v>
+      </c>
+      <c r="F202" s="28" t="s">
+        <v>101</v>
+      </c>
+      <c r="G202" s="30">
+        <v>112</v>
+      </c>
+      <c r="H202" s="30" t="s">
+        <v>448</v>
+      </c>
+      <c r="I202" s="32" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A203" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="B203" s="29">
+        <v>46269</v>
+      </c>
+      <c r="C203" s="29">
+        <v>46269</v>
+      </c>
+      <c r="D203" s="29">
+        <v>46330</v>
+      </c>
+      <c r="E203" s="28" t="s">
+        <v>449</v>
+      </c>
+      <c r="F203" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="G203" s="30">
+        <v>176</v>
+      </c>
+      <c r="H203" s="30" t="s">
+        <v>450</v>
+      </c>
+      <c r="I203" s="32" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -8781,7 +9095,7 @@
           <x14:formula1>
             <xm:f>'Industry List'!$A$1:$A$22</xm:f>
           </x14:formula1>
-          <xm:sqref>I3:I194</xm:sqref>
+          <xm:sqref>I3:I203</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -8902,7 +9216,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="99.75" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
-        <v>420</v>
+        <v>431</v>
       </c>
       <c r="E1"/>
     </row>
@@ -9317,7 +9631,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76B6A9E8-AD51-41FA-8B02-23E48CE4D608}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D66BF66C-BF6C-4375-A98D-BFB3C8F7CBF2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -9336,7 +9650,7 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA7AD1B3-404A-4EEA-9271-4F03D692E459}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AA4052B-B7DB-426A-99A3-3ADFC19DC050}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
@@ -9344,24 +9658,24 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39B02763-705B-493C-839B-26A069D90AFA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFC42A0E-256F-48F9-A375-77C39F1E4474}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="82b749e3-8208-459a-bfc0-9b428d09cbab"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="9ac7e9dd-8d2d-4750-b54a-f534515ac3a2"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{651480e4-deb2-4da5-bc64-7d1e9e1df8e4}" enabled="1" method="Standard" siteId="{06cac249-57c6-4eed-94fd-256abde82b4e}" contentBits="0" removed="0"/>
+  <clbl:label id="{651480e4-deb2-4da5-bc64-7d1e9e1df8e4}" enabled="1" method="Standard" siteId="{06cac249-57c6-4eed-94fd-256abde82b4e}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>